<commit_message>
Initialize GST ITC Reconciliation App with GSTR-3B Classification and empty template
- Implemented GSTR-3B Table 4 classification logic (4A5, 4B1, 4B2, 4C) in the backend.
- Updated FastAPI models and schemas to support sub-status and common ITC flags.
- Enhanced Excel parsing to handle flexible headers and clean formatted numeric strings.
- Refined React dashboard with a GSTR-3B summary table and improved invoice management.
- Added empty Excel template 'test_data.xlsx' with required headers.
- Verified functionality with Playwright and comprehensive backend testing.

Co-authored-by: caaravindguru <265460247+caaravindguru@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -413,18 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Mont</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Particular</t>
+          <t>Particulars</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -475,110 +475,6 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Apr-24</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GSTR2B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>03AAACQ3814D1Z2</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>V-CON</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1802460051</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>03/04/2024</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>18</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2259465.9</v>
-      </c>
-      <c r="I2" t="n">
-        <v>406703.87</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Apr-24</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GSTR2B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>07AAAFF0686K2ZB</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FILMISTAN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>24056</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>09/04/2024</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>18</v>
-      </c>
-      <c r="H3" t="n">
-        <v>81300</v>
-      </c>
-      <c r="I3" t="n">
-        <v>14634</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Not in books</t>
         </is>
       </c>
     </row>

</xml_diff>